<commit_message>
test: adiciona suíte automatizada no backend (US-15)
- Jest + Supertest cobrindo alimentos, categorias e relatórios (30 testes, 3 suítes)
- pool do pg mockado nos testes, sem depender de conexão real com o banco
- server.js exporta o app e só sobe o servidor quando executado diretamente
- README, ProductBacklog e SprintBacklog atualizados com o status da US-15
</commit_message>
<xml_diff>
--- a/docs/ReFood_ProductBacklog.xlsx
+++ b/docs/ReFood_ProductBacklog.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="164">
   <si>
     <t xml:space="preserve">🌿  ReFood  —  Product Backlog</t>
   </si>
@@ -342,7 +342,7 @@
     <t xml:space="preserve">Como equipe, queremos testes automatizados no backend para garantir que mudanças futuras não quebrem funcionalidades existentes.</t>
   </si>
   <si>
-    <t xml:space="preserve">Suíte Jest + Supertest cobrindo os endpoints de alimentos e categorias; script npm test funcional; roda contra uma branch de banco isolada no Neon</t>
+    <t xml:space="preserve">Suíte Jest + Supertest cobrindo os endpoints de alimentos, categorias e relatórios (30 testes, 3 suítes); script npm test funcional; roda com o pool do pg mockado, sem depender de conexão real com o banco.</t>
   </si>
   <si>
     <t xml:space="preserve">RNF-06</t>
@@ -351,7 +351,10 @@
     <t xml:space="preserve">Equipe</t>
   </si>
   <si>
-    <t xml:space="preserve">Nova story — não existia no backlog original (equipe de 4 pessoas não tinha essa frente listada).</t>
+    <t xml:space="preserve">Concluído (backend)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Entregue: backend/tests/ (helpers/mockPool.js + alimentos/categorias/relatorios.test.js). server.js ajustado pra exportar o app sem subir servidor durante os testes.</t>
   </si>
   <si>
     <t xml:space="preserve">TOTAL DE STORY POINTS</t>
@@ -2136,16 +2139,16 @@
       <c r="H25" s="26" t="s">
         <v>108</v>
       </c>
-      <c r="I25" s="27" t="s">
-        <v>76</v>
+      <c r="I25" s="36" t="s">
+        <v>109</v>
       </c>
       <c r="J25" s="28" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="43" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B26" s="43"/>
       <c r="C26" s="43"/>
@@ -2206,7 +2209,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="46" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B1" s="46"/>
       <c r="C1" s="46"/>
@@ -2216,7 +2219,7 @@
     </row>
     <row r="2" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="47" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B2" s="47"/>
       <c r="C2" s="47"/>
@@ -2237,10 +2240,10 @@
         <v>15</v>
       </c>
       <c r="B4" s="48" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C4" s="48" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D4" s="48" t="s">
         <v>17</v>
@@ -2249,107 +2252,107 @@
         <v>19</v>
       </c>
       <c r="F4" s="48" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="49" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B5" s="50" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C5" s="22" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D5" s="22" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="E5" s="23" t="s">
         <v>29</v>
       </c>
       <c r="F5" s="38" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="51" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B6" s="52" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C6" s="31" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D6" s="31" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E6" s="23" t="s">
         <v>29</v>
       </c>
       <c r="F6" s="38" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="49" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B7" s="50" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C7" s="22" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D7" s="22" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="E7" s="23" t="s">
         <v>29</v>
       </c>
       <c r="F7" s="38" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="51" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B8" s="52" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C8" s="31" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D8" s="31" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="E8" s="23" t="s">
         <v>29</v>
       </c>
       <c r="F8" s="38" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="49" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B9" s="50" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C9" s="22" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D9" s="22" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="E9" s="35" t="s">
         <v>42</v>
       </c>
       <c r="F9" s="38" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2357,19 +2360,19 @@
         <v>107</v>
       </c>
       <c r="B10" s="52" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C10" s="31" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D10" s="31" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="E10" s="41" t="s">
         <v>101</v>
       </c>
       <c r="F10" s="38" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
   </sheetData>
@@ -2407,7 +2410,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="53" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B1" s="53"/>
       <c r="C1" s="53"/>
@@ -2417,7 +2420,7 @@
     </row>
     <row r="2" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -2438,7 +2441,7 @@
         <v>21</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C4" s="19" t="s">
         <v>8</v>
@@ -2447,7 +2450,7 @@
         <v>12</v>
       </c>
       <c r="E4" s="19" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="F4" s="19" t="s">
         <v>24</v>
@@ -2458,10 +2461,10 @@
         <v>30</v>
       </c>
       <c r="B5" s="50" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D5" s="54" t="n">
         <v>19</v>
@@ -2471,7 +2474,7 @@
         <v>0.327586206896552</v>
       </c>
       <c r="F5" s="22" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2479,10 +2482,10 @@
         <v>75</v>
       </c>
       <c r="B6" s="50" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C6" s="21" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D6" s="54" t="n">
         <v>13</v>
@@ -2492,7 +2495,7 @@
         <v>0.224137931034483</v>
       </c>
       <c r="F6" s="22" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2500,10 +2503,10 @@
         <v>81</v>
       </c>
       <c r="B7" s="50" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C7" s="21" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D7" s="54" t="n">
         <v>16</v>
@@ -2513,7 +2516,7 @@
         <v>0.275862068965517</v>
       </c>
       <c r="F7" s="22" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2521,10 +2524,10 @@
         <v>102</v>
       </c>
       <c r="B8" s="50" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C8" s="21" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D8" s="54" t="n">
         <v>16</v>
@@ -2534,12 +2537,12 @@
         <v>0.275862068965517</v>
       </c>
       <c r="F8" s="22" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="43" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B9" s="43"/>
       <c r="C9" s="43"/>
@@ -2555,7 +2558,7 @@
     </row>
     <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="57" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B11" s="57"/>
       <c r="C11" s="57"/>

</xml_diff>